<commit_message>
#30 Centroid File Format updated.
</commit_message>
<xml_diff>
--- a/BOM Format/BOM Template/Centroid File-JLCPCB.xlsx
+++ b/BOM Format/BOM Template/Centroid File-JLCPCB.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\eSpark-Hardware\BOM Format\BOM Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60518A2C-6B03-479D-A566-A503C8ED8B92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5298C9-D8D4-495B-A8A7-91C7CE702F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Column=Rotation</t>
   </si>
   <si>
-    <t>Note : File Formate CSV hoga or Comma , Seprated File generate hogi, Units mention ni honge file me,  Column Names Change krne han , Layer k Column me jo Value ayegi us k Sath Layer ni ana chahiye.</t>
+    <t>Note : File Formate CSV hoga or Dot . Seprated File generate hogi, Units mm honge file me,  Column Names Change krne han , Layer k Column me jo Value ayegi us k Sath Layer ni ana chahiye.</t>
   </si>
 </sst>
 </file>
@@ -631,7 +631,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="6" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
         <v>5</v>
       </c>

</xml_diff>